<commit_message>
Article 43 initial publish; tweaks to No.42
</commit_message>
<xml_diff>
--- a/articles/43-does-this-decision-need-an-llm/templates/decision_model_pilot_worksheet.xlsx
+++ b/articles/43-does-this-decision-need-an-llm/templates/decision_model_pilot_worksheet.xlsx
@@ -631,7 +631,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>6. For every wrong answer, record how bad it would have been: annoying (wrong queue, a person catches it), costly (delay, rework), or control failure (cleared with no review).</t>
+          <t>6. For every wrong answer, record how bad it would have been: minor (wrong queue, a person catches it), costly (delay, rework), or control failure (cleared with no review).</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>annoying</t>
+          <t>minor</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>annoying</t>
+          <t>minor</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
@@ -1808,7 +1808,7 @@
       <formula1>"cash_flow,pricing_dispute,purchase_order,quantity_dispute,other"</formula1>
     </dataValidation>
     <dataValidation sqref="I5:I24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"annoying,costly,control failure"</formula1>
+      <formula1>"minor,costly,control failure"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2668,7 +2668,7 @@
       <formula1>"cash_flow,pricing_dispute,purchase_order,quantity_dispute,other"</formula1>
     </dataValidation>
     <dataValidation sqref="I5:I29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"annoying,costly,control failure"</formula1>
+      <formula1>"minor,costly,control failure"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>